<commit_message>
fix: dashboard bugs + menu update from Shree Radhe Radhe Menu Rates
- Fixed FieldError: is_occupied field does not exist on RestaurantTable
  (replaced with status=TableStatus.OCCUPIED/BILLED query)
- Fixed order_order_by typo in get_daily_report -> .order_by()
- Added TableStatus + RestaurantSettings imports to services.py
- Updated radhe_sweets_menu: 201 items across 18 categories (merged
  Shree_Radhe_Radhe_Menu_Rates new items with existing menu)
</commit_message>
<xml_diff>
--- a/radhe_sweets_menu.xlsx
+++ b/radhe_sweets_menu.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2369,12 +2369,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Poori Sabji - 4 Pc</t>
+          <t>Steam Veg Momos</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2382,21 +2382,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr"/>
+      <c r="D87" t="n">
+        <v>80</v>
+      </c>
       <c r="E87" t="n">
-        <v>80</v>
-      </c>
-      <c r="F87" t="inlineStr"/>
+        <v>110</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Chole + Plain Bhature</t>
+          <t>Fried Veg Momos</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2404,21 +2410,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr"/>
+      <c r="D88" t="n">
+        <v>90</v>
+      </c>
       <c r="E88" t="n">
-        <v>80</v>
-      </c>
-      <c r="F88" t="inlineStr"/>
+        <v>130</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Chole + Paneer Bhature</t>
+          <t>Kurkure Veg Momos</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2426,21 +2438,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr"/>
+      <c r="D89" t="n">
+        <v>99</v>
+      </c>
       <c r="E89" t="n">
-        <v>100</v>
-      </c>
-      <c r="F89" t="inlineStr"/>
+        <v>140</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Aloo Paratha with Curd -1 Pce</t>
+          <t>Tandoori Veg Momos</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2448,21 +2466,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr"/>
+      <c r="D90" t="n">
+        <v>100</v>
+      </c>
       <c r="E90" t="n">
-        <v>100</v>
-      </c>
-      <c r="F90" t="inlineStr"/>
+        <v>160</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Gobhi Paratha with Curd -1 Pcs</t>
+          <t>Chilli Dry Veg Momos</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2470,21 +2494,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr"/>
+      <c r="D91" t="n">
+        <v>110</v>
+      </c>
       <c r="E91" t="n">
-        <v>120</v>
-      </c>
-      <c r="F91" t="inlineStr"/>
+        <v>170</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Mix Veg Paratha with Curd - 1 Pcs</t>
+          <t>Tandoori Veg Malai Momos</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2492,21 +2522,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr"/>
+      <c r="D92" t="n">
+        <v>130</v>
+      </c>
       <c r="E92" t="n">
-        <v>120</v>
-      </c>
-      <c r="F92" t="inlineStr"/>
+        <v>200</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Breakfast</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Paneer Paratha with Curd - 1 Pcs</t>
+          <t>Steam Paneer Momos</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2514,21 +2550,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr"/>
+      <c r="D93" t="n">
+        <v>100</v>
+      </c>
       <c r="E93" t="n">
-        <v>150</v>
-      </c>
-      <c r="F93" t="inlineStr"/>
+        <v>160</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Plain Dosa</t>
+          <t>Fried Paneer Momos</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2536,21 +2578,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="n">
+        <v>110</v>
+      </c>
       <c r="E94" t="n">
-        <v>120</v>
-      </c>
-      <c r="F94" t="inlineStr"/>
+        <v>170</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Masala Dosa</t>
+          <t>Kurkure Paneer Momos</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2558,21 +2606,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="n">
+        <v>119</v>
+      </c>
       <c r="E95" t="n">
-        <v>140</v>
-      </c>
-      <c r="F95" t="inlineStr"/>
+        <v>190</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Butter Plain Dosa</t>
+          <t>Tandoori Paneer Momos</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2580,21 +2634,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr"/>
+      <c r="D96" t="n">
+        <v>120</v>
+      </c>
       <c r="E96" t="n">
-        <v>150</v>
-      </c>
-      <c r="F96" t="inlineStr"/>
+        <v>210</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Butter Masala Dosa</t>
+          <t>Chilli Dry Paneer Momos</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2602,21 +2662,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr"/>
+      <c r="D97" t="n">
+        <v>130</v>
+      </c>
       <c r="E97" t="n">
-        <v>180</v>
-      </c>
-      <c r="F97" t="inlineStr"/>
+        <v>230</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chalo Momos Khate Hai</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Paneer Plain Dosa</t>
+          <t>Tandoori Paneer Malai Momos</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2624,21 +2690,27 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr"/>
+      <c r="D98" t="n">
+        <v>160</v>
+      </c>
       <c r="E98" t="n">
-        <v>160</v>
-      </c>
-      <c r="F98" t="inlineStr"/>
+        <v>240</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>4 Pcs / 8 Pcs</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chinese Sizzler Combo</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Paneer Masala Dosa</t>
+          <t>Fried Rice + Veg Manchurian</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2648,19 +2720,19 @@
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chinese Sizzler Combo</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Paneer Butter Masala Dosa</t>
+          <t>Fried Rice + Paneer Manchurian</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2677,12 +2749,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chinese Sizzler Combo</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Cheese Plain Dosa</t>
+          <t>Garlic Noodles + Veg Manchurian</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2692,19 +2764,19 @@
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chinese Sizzler Combo</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Cheese Masala Dosa</t>
+          <t>Schezwan Fried Rice + Paneer Chili Gravy</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2714,19 +2786,19 @@
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Chinese Sizzler Combo</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Rava Dosa</t>
+          <t>Noodles with chilli Paneer</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2736,19 +2808,19 @@
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Rava Masala Dosa</t>
+          <t>Poori Sabji - 4 Pc</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2758,19 +2830,19 @@
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Rava Cheese Dosa</t>
+          <t>Chole + Plain Bhature</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2780,19 +2852,19 @@
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="n">
-        <v>220</v>
+        <v>80</v>
       </c>
       <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Rava Butter Paneer Dosa</t>
+          <t>Chole + Paneer Bhature</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2802,19 +2874,19 @@
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="n">
-        <v>240</v>
+        <v>100</v>
       </c>
       <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Schezwan masala Dosa</t>
+          <t>Aloo Paratha with Curd</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2824,19 +2896,19 @@
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="n">
-        <v>240</v>
+        <v>100</v>
       </c>
       <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Radhe Radhe Special dosa</t>
+          <t>Gobhi Paratha with Curd</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2846,19 +2918,19 @@
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sambhar Vada -2 Pcs</t>
+          <t>Mix Veg Paratha with Curd</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2868,19 +2940,19 @@
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>South Indian</t>
+          <t>Breakfast</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Idli Sambhar -2 Pcs</t>
+          <t>Paneer Paratha with Curd</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2890,7 +2962,7 @@
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="F110" t="inlineStr"/>
     </row>
@@ -2902,7 +2974,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Fry Idli - 2 Pcs</t>
+          <t>Plain Dosa</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2924,7 +2996,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Masala Uttapam</t>
+          <t>Masala Dosa</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2934,7 +3006,7 @@
       </c>
       <c r="D112" t="inlineStr"/>
       <c r="E112" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="F112" t="inlineStr"/>
     </row>
@@ -2946,7 +3018,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Onion Uttapam</t>
+          <t>Butter Plain Dosa</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2956,7 +3028,7 @@
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="n">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="F113" t="inlineStr"/>
     </row>
@@ -2968,7 +3040,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Mix Uttapam</t>
+          <t>Butter Masala Dosa</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2990,7 +3062,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>South Indian Thali (mini dosa + Mini Uttapam + Idli)</t>
+          <t>Paneer Plain Dosa</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3000,19 +3072,19 @@
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="n">
-        <v>300</v>
+        <v>160</v>
       </c>
       <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Steam Veg Momos</t>
+          <t>Paneer Masala Dosa</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3020,27 +3092,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D116" t="n">
-        <v>80</v>
-      </c>
+      <c r="D116" t="inlineStr"/>
       <c r="E116" t="n">
-        <v>110</v>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Fried Veg Momos</t>
+          <t>Paneer Butter Masala Dosa</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -3048,27 +3114,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D117" t="n">
-        <v>90</v>
-      </c>
+      <c r="D117" t="inlineStr"/>
       <c r="E117" t="n">
-        <v>130</v>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>230</v>
+      </c>
+      <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Kurkure Veg Momos</t>
+          <t>Cheese Plain Dosa</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3076,27 +3136,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D118" t="n">
-        <v>99</v>
-      </c>
+      <c r="D118" t="inlineStr"/>
       <c r="E118" t="n">
-        <v>140</v>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tandoori Veg Momos</t>
+          <t>Cheese Masala Dosa</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3104,27 +3158,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D119" t="n">
-        <v>100</v>
-      </c>
+      <c r="D119" t="inlineStr"/>
       <c r="E119" t="n">
-        <v>160</v>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Chilli Dry Veg Momos</t>
+          <t>Rava Dosa</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3132,27 +3180,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D120" t="n">
-        <v>110</v>
-      </c>
+      <c r="D120" t="inlineStr"/>
       <c r="E120" t="n">
-        <v>170</v>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>180</v>
+      </c>
+      <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Tandoori Veg Malai Momos</t>
+          <t>Rava Masala Dosa</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3160,27 +3202,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D121" t="n">
-        <v>130</v>
-      </c>
+      <c r="D121" t="inlineStr"/>
       <c r="E121" t="n">
         <v>200</v>
       </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+      <c r="F121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Steam Paneer Momos</t>
+          <t>Rava Cheese Dosa</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3188,27 +3224,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D122" t="n">
-        <v>100</v>
-      </c>
+      <c r="D122" t="inlineStr"/>
       <c r="E122" t="n">
-        <v>160</v>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>220</v>
+      </c>
+      <c r="F122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Fried Paneer Momos</t>
+          <t>Rava Butter Paneer Dosa</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3216,27 +3246,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D123" t="n">
-        <v>110</v>
-      </c>
+      <c r="D123" t="inlineStr"/>
       <c r="E123" t="n">
-        <v>170</v>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Kurkure Paneer Momos</t>
+          <t>Schezwan Masala Dosa</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3244,27 +3268,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D124" t="n">
-        <v>119</v>
-      </c>
+      <c r="D124" t="inlineStr"/>
       <c r="E124" t="n">
-        <v>190</v>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>240</v>
+      </c>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Tandoori Paneer Momos</t>
+          <t>Radhe Radhe Special Dosa</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3272,27 +3290,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D125" t="n">
-        <v>120</v>
-      </c>
+      <c r="D125" t="inlineStr"/>
       <c r="E125" t="n">
-        <v>210</v>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Chilli Dry Paneer Momos</t>
+          <t>Sambhar Vada (2)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3300,27 +3312,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D126" t="n">
-        <v>130</v>
-      </c>
+      <c r="D126" t="inlineStr"/>
       <c r="E126" t="n">
-        <v>230</v>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Chalo Momos Khate Hai</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Tandoori Paneer Malai Momos</t>
+          <t>Idli Sambhar (2)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3328,27 +3334,21 @@
           <t>Veg</t>
         </is>
       </c>
-      <c r="D127" t="n">
-        <v>160</v>
-      </c>
+      <c r="D127" t="inlineStr"/>
       <c r="E127" t="n">
-        <v>240</v>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>4 Pcs / 8 Pcs</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Chinese Sizzler Combo</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Fried Rice + Veg Manchurian</t>
+          <t>Fry Idli (2)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3358,19 +3358,19 @@
       </c>
       <c r="D128" t="inlineStr"/>
       <c r="E128" t="n">
-        <v>215</v>
+        <v>120</v>
       </c>
       <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Chinese Sizzler Combo</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Fried Rice + Paneer Manchurian</t>
+          <t>Masala Uttapam</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3380,19 +3380,19 @@
       </c>
       <c r="D129" t="inlineStr"/>
       <c r="E129" t="n">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Chinese Sizzler Combo</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Garlic Noodles + Veg Manchurian</t>
+          <t>Onion Uttapam</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3402,19 +3402,19 @@
       </c>
       <c r="D130" t="inlineStr"/>
       <c r="E130" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Chinese Sizzler Combo</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Schezwan Fried Rice + Paneer Chili Gravy</t>
+          <t>Mix Uttapam</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -3424,19 +3424,19 @@
       </c>
       <c r="D131" t="inlineStr"/>
       <c r="E131" t="n">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Chinese Sizzler Combo</t>
+          <t>South Indian</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Noodles with chilli Paneer</t>
+          <t>South Indian Thali</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3446,9 +3446,1589 @@
       </c>
       <c r="D132" t="inlineStr"/>
       <c r="E132" t="n">
-        <v>230</v>
+        <v>300</v>
       </c>
       <c r="F132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Tandoori Plain Roti</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="n">
+        <v>20</v>
+      </c>
+      <c r="F133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Tandoori Butter Roti</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="n">
+        <v>25</v>
+      </c>
+      <c r="F134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Plain Tawa Roti</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="n">
+        <v>15</v>
+      </c>
+      <c r="F135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Butter Tawa Roti</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="n">
+        <v>20</v>
+      </c>
+      <c r="F136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Missi Roti</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="n">
+        <v>50</v>
+      </c>
+      <c r="F137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Lachha Paratha</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="n">
+        <v>55</v>
+      </c>
+      <c r="F138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Cheese Chilli Paratha</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="n">
+        <v>100</v>
+      </c>
+      <c r="F139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Plain Kulcha</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="n">
+        <v>50</v>
+      </c>
+      <c r="F140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Onion Kulcha</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="n">
+        <v>100</v>
+      </c>
+      <c r="F141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Masala Kulcha</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="n">
+        <v>100</v>
+      </c>
+      <c r="F142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Amritsari Kulcha</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="n">
+        <v>100</v>
+      </c>
+      <c r="F143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Aloo Kulcha</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="n">
+        <v>80</v>
+      </c>
+      <c r="F144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Paneer Kulcha</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="n">
+        <v>120</v>
+      </c>
+      <c r="F145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Plain Naan</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="n">
+        <v>50</v>
+      </c>
+      <c r="F146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Butter Naan</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="n">
+        <v>60</v>
+      </c>
+      <c r="F147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Garlic Naan</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="n">
+        <v>100</v>
+      </c>
+      <c r="F148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Kashmiri Naan</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="n">
+        <v>150</v>
+      </c>
+      <c r="F149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Cheese Naan</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="n">
+        <v>120</v>
+      </c>
+      <c r="F150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Cheese Chilli Garlic Naan</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="n">
+        <v>150</v>
+      </c>
+      <c r="F151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Stuffed Naan</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="n">
+        <v>100</v>
+      </c>
+      <c r="F152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Bread &amp; Roti</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Shree Radhe Radhe Spl. Kulcha</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="n">
+        <v>150</v>
+      </c>
+      <c r="F153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Indian Combo</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Mix Veg, Jeera Rice &amp; Dal Combo</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="n">
+        <v>180</v>
+      </c>
+      <c r="F154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Indian Combo</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Dal Makhni, Veg Pulao &amp; Roti (2)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="n">
+        <v>200</v>
+      </c>
+      <c r="F155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Indian Combo</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Shahi Paneer + 1 Butter Naan +1 Roti</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="n">
+        <v>200</v>
+      </c>
+      <c r="F156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Thali</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Bahubali Thali</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="n">
+        <v>350</v>
+      </c>
+      <c r="F157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Thali</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Shree Radhe Radhe Spl. Thali</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="n">
+        <v>380</v>
+      </c>
+      <c r="F158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Lemon Tea</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="n">
+        <v>30</v>
+      </c>
+      <c r="F159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Black Tea</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="n">
+        <v>40</v>
+      </c>
+      <c r="F160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Ice Tea</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="n">
+        <v>60</v>
+      </c>
+      <c r="F161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Milk Tea</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="n">
+        <v>50</v>
+      </c>
+      <c r="F162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Hot Coffee</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="n">
+        <v>60</v>
+      </c>
+      <c r="F163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Hot Beverage</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Espresso Coffee</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="n">
+        <v>60</v>
+      </c>
+      <c r="F164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Sweet Lassi</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="n">
+        <v>99</v>
+      </c>
+      <c r="F165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Salted Lassi</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="n">
+        <v>99</v>
+      </c>
+      <c r="F166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Mango Lassi</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="n">
+        <v>170</v>
+      </c>
+      <c r="F167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Strawberry Lassi</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="n">
+        <v>180</v>
+      </c>
+      <c r="F168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Chocolate Lassi</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="n">
+        <v>190</v>
+      </c>
+      <c r="F169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Butter Milk</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="n">
+        <v>69</v>
+      </c>
+      <c r="F170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Lassi</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Masala Butter Milk</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="n">
+        <v>99</v>
+      </c>
+      <c r="F171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Spicy Mango</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="n">
+        <v>99</v>
+      </c>
+      <c r="F172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Virgin Mojito</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="n">
+        <v>99</v>
+      </c>
+      <c r="F173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Red Litchi Dragon</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="n">
+        <v>109</v>
+      </c>
+      <c r="F174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Red Rose</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
+      <c r="E175" t="n">
+        <v>109</v>
+      </c>
+      <c r="F175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="n">
+        <v>89</v>
+      </c>
+      <c r="F176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Blue Lagoon</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="n">
+        <v>99</v>
+      </c>
+      <c r="F177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Watermelon</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="n">
+        <v>79</v>
+      </c>
+      <c r="F178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Kiwi</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="n">
+        <v>109</v>
+      </c>
+      <c r="F179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Jamun Shot</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="n">
+        <v>139</v>
+      </c>
+      <c r="F180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Black Current</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="n">
+        <v>139</v>
+      </c>
+      <c r="F181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Green Apple</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr"/>
+      <c r="E182" t="n">
+        <v>130</v>
+      </c>
+      <c r="F182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Aam Panna</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="n">
+        <v>110</v>
+      </c>
+      <c r="F183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Tango Mango</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="n">
+        <v>140</v>
+      </c>
+      <c r="F184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Mocktail</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Banta Soda</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="n">
+        <v>90</v>
+      </c>
+      <c r="F185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Cold Coffee</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="n">
+        <v>79</v>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Cold Coffee With Icecream</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="n">
+        <v>109</v>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Vanilla Milk Shake</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="n">
+        <v>99</v>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Strawberry Milk Shake</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="n">
+        <v>109</v>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Butter Scotch Shake</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="n">
+        <v>109</v>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Oreo Shake</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="n">
+        <v>109</v>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Kitkat Shake</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="n">
+        <v>109</v>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Chocolate Shake</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="n">
+        <v>99</v>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Masala Colddrink</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="n">
+        <v>80</v>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Cold Beverages</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Mix Fruit Punch</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="n">
+        <v>149</v>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>MRP items excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Veg Sweet Corn Soup</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="n">
+        <v>109</v>
+      </c>
+      <c r="F196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Veg Munchow Soup</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="n">
+        <v>109</v>
+      </c>
+      <c r="F197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Veg Hot &amp; Sour Soup</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="n">
+        <v>109</v>
+      </c>
+      <c r="F198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Veg Lemon Corriander Soup</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="n">
+        <v>129</v>
+      </c>
+      <c r="F199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Cream of Tomato Soup</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="n">
+        <v>109</v>
+      </c>
+      <c r="F200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Cream of Mushroom Soup</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+      <c r="E201" t="n">
+        <v>119</v>
+      </c>
+      <c r="F201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Soup</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Shree Radhe Radhe Soup</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Veg</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="n">
+        <v>120</v>
+      </c>
+      <c r="F202" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>